<commit_message>
Fix imageURL function with full public URLs
</commit_message>
<xml_diff>
--- a/Summer-Camp-Quick-Summary.xlsx
+++ b/Summer-Camp-Quick-Summary.xlsx
@@ -779,13 +779,13 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H6">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I6">
         <v>2</v>

</xml_diff>